<commit_message>
implemented  density and EPD-backed carbon calculation (B2) and updating of visualization
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -971,9 +971,7 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="Y4" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="Y4" s="7" t="n"/>
       <c r="AB4" s="7" t="inlineStr">
         <is>
           <t>2.8</t>
@@ -1055,9 +1053,7 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="Y5" s="7" t="n">
-        <v>248623</v>
-      </c>
+      <c r="Y5" s="7" t="n"/>
       <c r="AB5" s="7" t="inlineStr">
         <is>
           <t>2.26</t>
@@ -1137,12 +1133,8 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="Y6" s="7" t="n">
-        <v>284321.5</v>
-      </c>
-      <c r="Z6" s="7" t="n">
-        <v>2.363</v>
-      </c>
+      <c r="Y6" s="7" t="n"/>
+      <c r="Z6" s="7" t="n"/>
       <c r="AB6" s="7" t="inlineStr">
         <is>
           <t>2.28</t>
@@ -1448,7 +1440,9 @@
       <c r="P9" s="8" t="n"/>
       <c r="Q9" s="8" t="n"/>
       <c r="R9" s="8" t="n"/>
-      <c r="S9" s="8" t="n"/>
+      <c r="S9" s="8" t="n">
+        <v>18400</v>
+      </c>
       <c r="T9" s="8" t="n"/>
       <c r="U9" s="8" t="n">
         <v>8</v>
@@ -1459,9 +1453,15 @@
         </is>
       </c>
       <c r="W9" s="8" t="n"/>
-      <c r="X9" s="8" t="n"/>
-      <c r="Y9" s="8" t="n"/>
-      <c r="Z9" s="8" t="n"/>
+      <c r="X9" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="Y9" s="8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="Z9" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA9" s="8" t="n"/>
       <c r="AB9" s="8" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
       <c r="AW9" s="8" t="n"/>
       <c r="AX9" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 1840.0 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,9 @@
       <c r="P10" s="8" t="n"/>
       <c r="Q10" s="8" t="n"/>
       <c r="R10" s="8" t="n"/>
-      <c r="S10" s="8" t="n"/>
+      <c r="S10" s="8" t="n">
+        <v>16790</v>
+      </c>
       <c r="T10" s="8" t="n"/>
       <c r="U10" s="8" t="n">
         <v>7.3</v>
@@ -1575,9 +1577,15 @@
         </is>
       </c>
       <c r="W10" s="8" t="n"/>
-      <c r="X10" s="8" t="n"/>
-      <c r="Y10" s="8" t="n"/>
-      <c r="Z10" s="8" t="n"/>
+      <c r="X10" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="Y10" s="8" t="n">
+        <v>1679</v>
+      </c>
+      <c r="Z10" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA10" s="8" t="n"/>
       <c r="AB10" s="8" t="inlineStr">
         <is>
@@ -1611,7 +1619,7 @@
       <c r="AW10" s="8" t="n"/>
       <c r="AX10" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 1679.0 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1688,9 @@
       <c r="P11" s="8" t="n"/>
       <c r="Q11" s="8" t="n"/>
       <c r="R11" s="8" t="n"/>
-      <c r="S11" s="8" t="n"/>
+      <c r="S11" s="8" t="n">
+        <v>230</v>
+      </c>
       <c r="T11" s="8" t="n"/>
       <c r="U11" s="8" t="n">
         <v>0.1</v>
@@ -1691,9 +1701,15 @@
         </is>
       </c>
       <c r="W11" s="8" t="n"/>
-      <c r="X11" s="8" t="n"/>
-      <c r="Y11" s="8" t="n"/>
-      <c r="Z11" s="8" t="n"/>
+      <c r="X11" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="Y11" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z11" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA11" s="8" t="n"/>
       <c r="AB11" s="8" t="inlineStr">
         <is>
@@ -1727,7 +1743,7 @@
       <c r="AW11" s="8" t="n"/>
       <c r="AX11" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 23.0 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1812,9 @@
       <c r="P12" s="8" t="n"/>
       <c r="Q12" s="8" t="n"/>
       <c r="R12" s="8" t="n"/>
-      <c r="S12" s="8" t="n"/>
+      <c r="S12" s="8" t="n">
+        <v>1324.8</v>
+      </c>
       <c r="T12" s="8" t="n"/>
       <c r="U12" s="8" t="n">
         <v>14.4</v>
@@ -1807,9 +1825,15 @@
         </is>
       </c>
       <c r="W12" s="8" t="n"/>
-      <c r="X12" s="8" t="n"/>
-      <c r="Y12" s="8" t="n"/>
-      <c r="Z12" s="8" t="n"/>
+      <c r="X12" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="Y12" s="8" t="n">
+        <v>132.48</v>
+      </c>
+      <c r="Z12" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA12" s="8" t="n"/>
       <c r="AB12" s="8" t="inlineStr">
         <is>
@@ -1843,7 +1867,7 @@
       <c r="AW12" s="8" t="n"/>
       <c r="AX12" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 132.48 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2048,9 @@
       <c r="P14" s="8" t="n"/>
       <c r="Q14" s="8" t="n"/>
       <c r="R14" s="8" t="n"/>
-      <c r="S14" s="8" t="n"/>
+      <c r="S14" s="8" t="n">
+        <v>27120</v>
+      </c>
       <c r="T14" s="8" t="n"/>
       <c r="U14" s="8" t="n">
         <v>11.3</v>
@@ -2035,9 +2061,15 @@
         </is>
       </c>
       <c r="W14" s="8" t="n"/>
-      <c r="X14" s="8" t="n"/>
-      <c r="Y14" s="8" t="n"/>
-      <c r="Z14" s="8" t="n"/>
+      <c r="X14" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="Y14" s="8" t="n">
+        <v>3254.4</v>
+      </c>
+      <c r="Z14" s="8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AA14" s="8" t="n"/>
       <c r="AB14" s="8" t="inlineStr">
         <is>
@@ -2071,7 +2103,7 @@
       <c r="AW14" s="8" t="n"/>
       <c r="AX14" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 3254.4 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2172,9 @@
       <c r="P15" s="8" t="n"/>
       <c r="Q15" s="8" t="n"/>
       <c r="R15" s="8" t="n"/>
-      <c r="S15" s="8" t="n"/>
+      <c r="S15" s="8" t="n">
+        <v>2400</v>
+      </c>
       <c r="T15" s="8" t="n"/>
       <c r="U15" s="8" t="n">
         <v>1</v>
@@ -2151,9 +2185,15 @@
         </is>
       </c>
       <c r="W15" s="8" t="n"/>
-      <c r="X15" s="8" t="n"/>
-      <c r="Y15" s="8" t="n"/>
-      <c r="Z15" s="8" t="n"/>
+      <c r="X15" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="Y15" s="8" t="n">
+        <v>288</v>
+      </c>
+      <c r="Z15" s="8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AA15" s="8" t="n"/>
       <c r="AB15" s="8" t="inlineStr">
         <is>
@@ -2187,7 +2227,7 @@
       <c r="AW15" s="8" t="n"/>
       <c r="AX15" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 288.0 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2296,9 @@
       <c r="P16" s="8" t="n"/>
       <c r="Q16" s="8" t="n"/>
       <c r="R16" s="8" t="n"/>
-      <c r="S16" s="8" t="n"/>
+      <c r="S16" s="8" t="n">
+        <v>1440</v>
+      </c>
       <c r="T16" s="8" t="n"/>
       <c r="U16" s="8" t="n">
         <v>0.6</v>
@@ -2267,9 +2309,15 @@
         </is>
       </c>
       <c r="W16" s="8" t="n"/>
-      <c r="X16" s="8" t="n"/>
-      <c r="Y16" s="8" t="n"/>
-      <c r="Z16" s="8" t="n"/>
+      <c r="X16" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="Y16" s="8" t="n">
+        <v>172.8</v>
+      </c>
+      <c r="Z16" s="8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AA16" s="8" t="n"/>
       <c r="AB16" s="8" t="inlineStr">
         <is>
@@ -2303,7 +2351,7 @@
       <c r="AW16" s="8" t="n"/>
       <c r="AX16" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 172.8 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2420,9 @@
       <c r="P17" s="8" t="n"/>
       <c r="Q17" s="8" t="n"/>
       <c r="R17" s="8" t="n"/>
-      <c r="S17" s="8" t="n"/>
+      <c r="S17" s="8" t="n">
+        <v>4080</v>
+      </c>
       <c r="T17" s="8" t="n"/>
       <c r="U17" s="8" t="n">
         <v>1.7</v>
@@ -2383,9 +2433,15 @@
         </is>
       </c>
       <c r="W17" s="8" t="n"/>
-      <c r="X17" s="8" t="n"/>
-      <c r="Y17" s="8" t="n"/>
-      <c r="Z17" s="8" t="n"/>
+      <c r="X17" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="Y17" s="8" t="n">
+        <v>489.6</v>
+      </c>
+      <c r="Z17" s="8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AA17" s="8" t="n"/>
       <c r="AB17" s="8" t="inlineStr">
         <is>
@@ -2419,7 +2475,7 @@
       <c r="AW17" s="8" t="n"/>
       <c r="AX17" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 489.6 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2544,9 @@
       <c r="P18" s="8" t="n"/>
       <c r="Q18" s="8" t="n"/>
       <c r="R18" s="8" t="n"/>
-      <c r="S18" s="8" t="n"/>
+      <c r="S18" s="8" t="n">
+        <v>240</v>
+      </c>
       <c r="T18" s="8" t="n"/>
       <c r="U18" s="8" t="n">
         <v>0.1</v>
@@ -2499,9 +2557,15 @@
         </is>
       </c>
       <c r="W18" s="8" t="n"/>
-      <c r="X18" s="8" t="n"/>
-      <c r="Y18" s="8" t="n"/>
-      <c r="Z18" s="8" t="n"/>
+      <c r="X18" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="Y18" s="8" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="Z18" s="8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AA18" s="8" t="n"/>
       <c r="AB18" s="8" t="inlineStr">
         <is>
@@ -2535,7 +2599,7 @@
       <c r="AW18" s="8" t="n"/>
       <c r="AX18" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 28.8 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2894,9 @@
       <c r="P21" s="8" t="n"/>
       <c r="Q21" s="8" t="n"/>
       <c r="R21" s="8" t="n"/>
-      <c r="S21" s="8" t="n"/>
+      <c r="S21" s="8" t="n">
+        <v>1920</v>
+      </c>
       <c r="T21" s="8" t="n"/>
       <c r="U21" s="8" t="n">
         <v>0.8</v>
@@ -2841,9 +2907,15 @@
         </is>
       </c>
       <c r="W21" s="8" t="n"/>
-      <c r="X21" s="8" t="n"/>
-      <c r="Y21" s="8" t="n"/>
-      <c r="Z21" s="8" t="n"/>
+      <c r="X21" s="8" t="n">
+        <v>2400</v>
+      </c>
+      <c r="Y21" s="8" t="n">
+        <v>230.4</v>
+      </c>
+      <c r="Z21" s="8" t="n">
+        <v>0.12</v>
+      </c>
       <c r="AA21" s="8" t="n"/>
       <c r="AB21" s="8" t="inlineStr">
         <is>
@@ -2877,7 +2949,7 @@
       <c r="AW21" s="8" t="n"/>
       <c r="AX21" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 230.4 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>
@@ -2946,7 +3018,9 @@
       <c r="P22" s="8" t="n"/>
       <c r="Q22" s="8" t="n"/>
       <c r="R22" s="8" t="n"/>
-      <c r="S22" s="8" t="n"/>
+      <c r="S22" s="8" t="n">
+        <v>32300</v>
+      </c>
       <c r="T22" s="8" t="n"/>
       <c r="U22" s="8" t="n">
         <v>17</v>
@@ -2957,9 +3031,15 @@
         </is>
       </c>
       <c r="W22" s="8" t="n"/>
-      <c r="X22" s="8" t="n"/>
-      <c r="Y22" s="8" t="n"/>
-      <c r="Z22" s="8" t="n"/>
+      <c r="X22" s="8" t="n">
+        <v>1900</v>
+      </c>
+      <c r="Y22" s="8" t="n">
+        <v>7752</v>
+      </c>
+      <c r="Z22" s="8" t="n">
+        <v>0.24</v>
+      </c>
       <c r="AA22" s="8" t="n"/>
       <c r="AB22" s="8" t="inlineStr">
         <is>
@@ -2993,7 +3073,7 @@
       <c r="AW22" s="8" t="n"/>
       <c r="AX22" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 7752.0 kg CO₂e (Indian Brick Industry average EPD; density from SP 64).</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3142,9 @@
       <c r="P23" s="8" t="n"/>
       <c r="Q23" s="8" t="n"/>
       <c r="R23" s="8" t="n"/>
-      <c r="S23" s="8" t="n"/>
+      <c r="S23" s="8" t="n">
+        <v>76570</v>
+      </c>
       <c r="T23" s="8" t="n"/>
       <c r="U23" s="8" t="n">
         <v>40.3</v>
@@ -3073,9 +3155,15 @@
         </is>
       </c>
       <c r="W23" s="8" t="n"/>
-      <c r="X23" s="8" t="n"/>
-      <c r="Y23" s="8" t="n"/>
-      <c r="Z23" s="8" t="n"/>
+      <c r="X23" s="8" t="n">
+        <v>1900</v>
+      </c>
+      <c r="Y23" s="8" t="n">
+        <v>18376.8</v>
+      </c>
+      <c r="Z23" s="8" t="n">
+        <v>0.24</v>
+      </c>
       <c r="AA23" s="8" t="n"/>
       <c r="AB23" s="8" t="inlineStr">
         <is>
@@ -3109,7 +3197,7 @@
       <c r="AW23" s="8" t="n"/>
       <c r="AX23" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 18376.8 kg CO₂e (Indian Brick Industry average EPD; density from SP 64).</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3266,9 @@
       <c r="P24" s="8" t="n"/>
       <c r="Q24" s="8" t="n"/>
       <c r="R24" s="8" t="n"/>
-      <c r="S24" s="8" t="n"/>
+      <c r="S24" s="8" t="n">
+        <v>1944.65</v>
+      </c>
       <c r="T24" s="8" t="n"/>
       <c r="U24" s="8" t="n">
         <v>8.9</v>
@@ -3189,9 +3279,15 @@
         </is>
       </c>
       <c r="W24" s="8" t="n"/>
-      <c r="X24" s="8" t="n"/>
-      <c r="Y24" s="8" t="n"/>
-      <c r="Z24" s="8" t="n"/>
+      <c r="X24" s="8" t="n">
+        <v>1900</v>
+      </c>
+      <c r="Y24" s="8" t="n">
+        <v>466.72</v>
+      </c>
+      <c r="Z24" s="8" t="n">
+        <v>0.24</v>
+      </c>
       <c r="AA24" s="8" t="n"/>
       <c r="AB24" s="8" t="inlineStr">
         <is>
@@ -3225,7 +3321,7 @@
       <c r="AW24" s="8" t="n"/>
       <c r="AX24" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 466.72 kg CO₂e (Indian Brick Industry average EPD; density from SP 64).</t>
         </is>
       </c>
     </row>
@@ -3294,7 +3390,9 @@
       <c r="P25" s="8" t="n"/>
       <c r="Q25" s="8" t="n"/>
       <c r="R25" s="8" t="n"/>
-      <c r="S25" s="8" t="n"/>
+      <c r="S25" s="8" t="n">
+        <v>1048.8</v>
+      </c>
       <c r="T25" s="8" t="n"/>
       <c r="U25" s="8" t="n">
         <v>4.8</v>
@@ -3305,9 +3403,15 @@
         </is>
       </c>
       <c r="W25" s="8" t="n"/>
-      <c r="X25" s="8" t="n"/>
-      <c r="Y25" s="8" t="n"/>
-      <c r="Z25" s="8" t="n"/>
+      <c r="X25" s="8" t="n">
+        <v>1900</v>
+      </c>
+      <c r="Y25" s="8" t="n">
+        <v>251.71</v>
+      </c>
+      <c r="Z25" s="8" t="n">
+        <v>0.24</v>
+      </c>
       <c r="AA25" s="8" t="n"/>
       <c r="AB25" s="8" t="inlineStr">
         <is>
@@ -3341,7 +3445,7 @@
       <c r="AW25" s="8" t="n"/>
       <c r="AX25" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 251.71 kg CO₂e (Indian Brick Industry average EPD; density from SP 64).</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3514,9 @@
       <c r="P26" s="8" t="n"/>
       <c r="Q26" s="8" t="n"/>
       <c r="R26" s="8" t="n"/>
-      <c r="S26" s="8" t="n"/>
+      <c r="S26" s="8" t="n">
+        <v>3933</v>
+      </c>
       <c r="T26" s="8" t="n"/>
       <c r="U26" s="8" t="n">
         <v>18</v>
@@ -3421,9 +3527,15 @@
         </is>
       </c>
       <c r="W26" s="8" t="n"/>
-      <c r="X26" s="8" t="n"/>
-      <c r="Y26" s="8" t="n"/>
-      <c r="Z26" s="8" t="n"/>
+      <c r="X26" s="8" t="n">
+        <v>1900</v>
+      </c>
+      <c r="Y26" s="8" t="n">
+        <v>943.92</v>
+      </c>
+      <c r="Z26" s="8" t="n">
+        <v>0.24</v>
+      </c>
       <c r="AA26" s="8" t="n"/>
       <c r="AB26" s="8" t="inlineStr">
         <is>
@@ -3457,7 +3569,7 @@
       <c r="AW26" s="8" t="n"/>
       <c r="AX26" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 943.92 kg CO₂e (Indian Brick Industry average EPD; density from SP 64).</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3634,9 @@
       <c r="P27" s="8" t="n"/>
       <c r="Q27" s="8" t="n"/>
       <c r="R27" s="8" t="n"/>
-      <c r="S27" s="8" t="n"/>
+      <c r="S27" s="8" t="n">
+        <v>2.45</v>
+      </c>
       <c r="T27" s="8" t="n"/>
       <c r="U27" s="8" t="n">
         <v>0.0035</v>
@@ -3533,9 +3647,15 @@
         </is>
       </c>
       <c r="W27" s="8" t="n"/>
-      <c r="X27" s="8" t="n"/>
-      <c r="Y27" s="8" t="n"/>
-      <c r="Z27" s="8" t="n"/>
+      <c r="X27" s="8" t="n">
+        <v>700</v>
+      </c>
+      <c r="Y27" s="8" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="Z27" s="8" t="n">
+        <v>0.35</v>
+      </c>
       <c r="AA27" s="8" t="n"/>
       <c r="AB27" s="8" t="inlineStr"/>
       <c r="AC27" s="8" t="n"/>
@@ -3565,7 +3685,7 @@
       <c r="AW27" s="8" t="n"/>
       <c r="AX27" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 0.86 kg CO₂e (Indian Forestry average EPD; density from IS 287).</t>
         </is>
       </c>
     </row>
@@ -3641,9 +3761,13 @@
         </is>
       </c>
       <c r="W28" s="8" t="n"/>
-      <c r="X28" s="8" t="n"/>
+      <c r="X28" s="8" t="n">
+        <v>700</v>
+      </c>
       <c r="Y28" s="8" t="n"/>
-      <c r="Z28" s="8" t="n"/>
+      <c r="Z28" s="8" t="n">
+        <v>0.35</v>
+      </c>
       <c r="AA28" s="8" t="n"/>
       <c r="AB28" s="8" t="inlineStr">
         <is>
@@ -3871,9 +3995,13 @@
         </is>
       </c>
       <c r="W30" s="8" t="n"/>
-      <c r="X30" s="8" t="n"/>
+      <c r="X30" s="8" t="n">
+        <v>700</v>
+      </c>
       <c r="Y30" s="8" t="n"/>
-      <c r="Z30" s="8" t="n"/>
+      <c r="Z30" s="8" t="n">
+        <v>0.35</v>
+      </c>
       <c r="AA30" s="8" t="n"/>
       <c r="AB30" s="8" t="inlineStr">
         <is>
@@ -3985,9 +4113,13 @@
         </is>
       </c>
       <c r="W31" s="8" t="n"/>
-      <c r="X31" s="8" t="n"/>
+      <c r="X31" s="8" t="n">
+        <v>7850</v>
+      </c>
       <c r="Y31" s="8" t="n"/>
-      <c r="Z31" s="8" t="n"/>
+      <c r="Z31" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA31" s="8" t="n"/>
       <c r="AB31" s="8" t="inlineStr">
         <is>
@@ -4099,9 +4231,13 @@
         </is>
       </c>
       <c r="W32" s="8" t="n"/>
-      <c r="X32" s="8" t="n"/>
+      <c r="X32" s="8" t="n">
+        <v>7850</v>
+      </c>
       <c r="Y32" s="8" t="n"/>
-      <c r="Z32" s="8" t="n"/>
+      <c r="Z32" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA32" s="8" t="n"/>
       <c r="AB32" s="8" t="inlineStr">
         <is>
@@ -4213,9 +4349,13 @@
         </is>
       </c>
       <c r="W33" s="8" t="n"/>
-      <c r="X33" s="8" t="n"/>
+      <c r="X33" s="8" t="n">
+        <v>2700</v>
+      </c>
       <c r="Y33" s="8" t="n"/>
-      <c r="Z33" s="8" t="n"/>
+      <c r="Z33" s="8" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AA33" s="8" t="n"/>
       <c r="AB33" s="8" t="inlineStr">
         <is>
@@ -4327,9 +4467,13 @@
         </is>
       </c>
       <c r="W34" s="8" t="n"/>
-      <c r="X34" s="8" t="n"/>
+      <c r="X34" s="8" t="n">
+        <v>2700</v>
+      </c>
       <c r="Y34" s="8" t="n"/>
-      <c r="Z34" s="8" t="n"/>
+      <c r="Z34" s="8" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AA34" s="8" t="n"/>
       <c r="AB34" s="8" t="inlineStr">
         <is>
@@ -4441,9 +4585,13 @@
         </is>
       </c>
       <c r="W35" s="8" t="n"/>
-      <c r="X35" s="8" t="n"/>
+      <c r="X35" s="8" t="n">
+        <v>2700</v>
+      </c>
       <c r="Y35" s="8" t="n"/>
-      <c r="Z35" s="8" t="n"/>
+      <c r="Z35" s="8" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AA35" s="8" t="n"/>
       <c r="AB35" s="8" t="inlineStr">
         <is>
@@ -4555,9 +4703,13 @@
         </is>
       </c>
       <c r="W36" s="8" t="n"/>
-      <c r="X36" s="8" t="n"/>
+      <c r="X36" s="8" t="n">
+        <v>2700</v>
+      </c>
       <c r="Y36" s="8" t="n"/>
-      <c r="Z36" s="8" t="n"/>
+      <c r="Z36" s="8" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AA36" s="8" t="n"/>
       <c r="AB36" s="8" t="inlineStr">
         <is>
@@ -4781,9 +4933,13 @@
         </is>
       </c>
       <c r="W38" s="8" t="n"/>
-      <c r="X38" s="8" t="n"/>
+      <c r="X38" s="8" t="n">
+        <v>7850</v>
+      </c>
       <c r="Y38" s="8" t="n"/>
-      <c r="Z38" s="8" t="n"/>
+      <c r="Z38" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA38" s="8" t="n"/>
       <c r="AB38" s="8" t="inlineStr">
         <is>
@@ -4895,9 +5051,13 @@
         </is>
       </c>
       <c r="W39" s="8" t="n"/>
-      <c r="X39" s="8" t="n"/>
+      <c r="X39" s="8" t="n">
+        <v>2700</v>
+      </c>
       <c r="Y39" s="8" t="n"/>
-      <c r="Z39" s="8" t="n"/>
+      <c r="Z39" s="8" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="AA39" s="8" t="n"/>
       <c r="AB39" s="8" t="inlineStr">
         <is>
@@ -5009,9 +5169,15 @@
         </is>
       </c>
       <c r="W40" s="8" t="n"/>
-      <c r="X40" s="8" t="n"/>
-      <c r="Y40" s="8" t="n"/>
-      <c r="Z40" s="8" t="n"/>
+      <c r="X40" s="8" t="n">
+        <v>7850</v>
+      </c>
+      <c r="Y40" s="8" t="n">
+        <v>122.1</v>
+      </c>
+      <c r="Z40" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA40" s="8" t="n"/>
       <c r="AB40" s="8" t="inlineStr">
         <is>
@@ -5045,7 +5211,7 @@
       <c r="AW40" s="8" t="n"/>
       <c r="AX40" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 122.1 kg CO₂e (Tata Steel India EPD; density from IS 808).</t>
         </is>
       </c>
     </row>
@@ -5123,9 +5289,15 @@
         </is>
       </c>
       <c r="W41" s="8" t="n"/>
-      <c r="X41" s="8" t="n"/>
-      <c r="Y41" s="8" t="n"/>
-      <c r="Z41" s="8" t="n"/>
+      <c r="X41" s="8" t="n">
+        <v>7850</v>
+      </c>
+      <c r="Y41" s="8" t="n">
+        <v>345.95</v>
+      </c>
+      <c r="Z41" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA41" s="8" t="n"/>
       <c r="AB41" s="8" t="inlineStr">
         <is>
@@ -5159,7 +5331,7 @@
       <c r="AW41" s="8" t="n"/>
       <c r="AX41" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 345.95 kg CO₂e (Tata Steel India EPD; density from IS 808).</t>
         </is>
       </c>
     </row>
@@ -5237,9 +5409,13 @@
         </is>
       </c>
       <c r="W42" s="8" t="n"/>
-      <c r="X42" s="8" t="n"/>
+      <c r="X42" s="8" t="n">
+        <v>7850</v>
+      </c>
       <c r="Y42" s="8" t="n"/>
-      <c r="Z42" s="8" t="n"/>
+      <c r="Z42" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA42" s="8" t="n"/>
       <c r="AB42" s="8" t="inlineStr">
         <is>
@@ -5353,9 +5529,13 @@
         </is>
       </c>
       <c r="W43" s="8" t="n"/>
-      <c r="X43" s="8" t="n"/>
+      <c r="X43" s="8" t="n">
+        <v>2300</v>
+      </c>
       <c r="Y43" s="8" t="n"/>
-      <c r="Z43" s="8" t="n"/>
+      <c r="Z43" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA43" s="8" t="n"/>
       <c r="AB43" s="8" t="inlineStr">
         <is>
@@ -5458,7 +5638,9 @@
       <c r="P44" s="8" t="n"/>
       <c r="Q44" s="8" t="n"/>
       <c r="R44" s="8" t="n"/>
-      <c r="S44" s="8" t="n"/>
+      <c r="S44" s="8" t="n">
+        <v>264</v>
+      </c>
       <c r="T44" s="8" t="n"/>
       <c r="U44" s="8" t="n">
         <v>11</v>
@@ -5469,9 +5651,15 @@
         </is>
       </c>
       <c r="W44" s="8" t="n"/>
-      <c r="X44" s="8" t="n"/>
-      <c r="Y44" s="8" t="n"/>
-      <c r="Z44" s="8" t="n"/>
+      <c r="X44" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y44" s="8" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="Z44" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA44" s="8" t="n"/>
       <c r="AB44" s="8" t="inlineStr">
         <is>
@@ -5505,7 +5693,7 @@
       <c r="AW44" s="8" t="n"/>
       <c r="AX44" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 39.6 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5758,9 @@
       <c r="P45" s="8" t="n"/>
       <c r="Q45" s="8" t="n"/>
       <c r="R45" s="8" t="n"/>
-      <c r="S45" s="8" t="n"/>
+      <c r="S45" s="8" t="n">
+        <v>360</v>
+      </c>
       <c r="T45" s="8" t="n"/>
       <c r="U45" s="8" t="n">
         <v>9</v>
@@ -5581,9 +5771,15 @@
         </is>
       </c>
       <c r="W45" s="8" t="n"/>
-      <c r="X45" s="8" t="n"/>
-      <c r="Y45" s="8" t="n"/>
-      <c r="Z45" s="8" t="n"/>
+      <c r="X45" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y45" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="Z45" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA45" s="8" t="n"/>
       <c r="AB45" s="8" t="inlineStr">
         <is>
@@ -5617,7 +5813,7 @@
       <c r="AW45" s="8" t="n"/>
       <c r="AX45" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 54.0 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -6020,7 +6216,9 @@
       <c r="P49" s="8" t="n"/>
       <c r="Q49" s="8" t="n"/>
       <c r="R49" s="8" t="n"/>
-      <c r="S49" s="8" t="n"/>
+      <c r="S49" s="8" t="n">
+        <v>1280</v>
+      </c>
       <c r="T49" s="8" t="n"/>
       <c r="U49" s="8" t="n">
         <v>32</v>
@@ -6031,9 +6229,15 @@
         </is>
       </c>
       <c r="W49" s="8" t="n"/>
-      <c r="X49" s="8" t="n"/>
-      <c r="Y49" s="8" t="n"/>
-      <c r="Z49" s="8" t="n"/>
+      <c r="X49" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y49" s="8" t="n">
+        <v>192</v>
+      </c>
+      <c r="Z49" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA49" s="8" t="n"/>
       <c r="AB49" s="8" t="inlineStr">
         <is>
@@ -6067,7 +6271,7 @@
       <c r="AW49" s="8" t="n"/>
       <c r="AX49" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 192.0 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -6149,9 +6353,13 @@
         </is>
       </c>
       <c r="W50" s="8" t="n"/>
-      <c r="X50" s="8" t="n"/>
+      <c r="X50" s="8" t="n">
+        <v>2300</v>
+      </c>
       <c r="Y50" s="8" t="n"/>
-      <c r="Z50" s="8" t="n"/>
+      <c r="Z50" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA50" s="8" t="n"/>
       <c r="AB50" s="8" t="inlineStr">
         <is>
@@ -6267,9 +6475,13 @@
         </is>
       </c>
       <c r="W51" s="8" t="n"/>
-      <c r="X51" s="8" t="n"/>
+      <c r="X51" s="8" t="n">
+        <v>2300</v>
+      </c>
       <c r="Y51" s="8" t="n"/>
-      <c r="Z51" s="8" t="n"/>
+      <c r="Z51" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA51" s="8" t="n"/>
       <c r="AB51" s="8" t="inlineStr">
         <is>
@@ -6381,9 +6593,13 @@
         </is>
       </c>
       <c r="W52" s="8" t="n"/>
-      <c r="X52" s="8" t="n"/>
+      <c r="X52" s="8" t="n">
+        <v>7200</v>
+      </c>
       <c r="Y52" s="8" t="n"/>
-      <c r="Z52" s="8" t="n"/>
+      <c r="Z52" s="8" t="n">
+        <v>2.1</v>
+      </c>
       <c r="AA52" s="8" t="n"/>
       <c r="AB52" s="8" t="inlineStr">
         <is>
@@ -6495,9 +6711,13 @@
         </is>
       </c>
       <c r="W53" s="8" t="n"/>
-      <c r="X53" s="8" t="n"/>
+      <c r="X53" s="8" t="n">
+        <v>7850</v>
+      </c>
       <c r="Y53" s="8" t="n"/>
-      <c r="Z53" s="8" t="n"/>
+      <c r="Z53" s="8" t="n">
+        <v>1.85</v>
+      </c>
       <c r="AA53" s="8" t="n"/>
       <c r="AB53" s="8" t="inlineStr">
         <is>
@@ -6609,9 +6829,13 @@
         </is>
       </c>
       <c r="W54" s="8" t="n"/>
-      <c r="X54" s="8" t="n"/>
+      <c r="X54" s="8" t="n">
+        <v>7200</v>
+      </c>
       <c r="Y54" s="8" t="n"/>
-      <c r="Z54" s="8" t="n"/>
+      <c r="Z54" s="8" t="n">
+        <v>2.1</v>
+      </c>
       <c r="AA54" s="8" t="n"/>
       <c r="AB54" s="8" t="inlineStr">
         <is>
@@ -6714,7 +6938,9 @@
       <c r="P55" s="8" t="n"/>
       <c r="Q55" s="8" t="n"/>
       <c r="R55" s="8" t="n"/>
-      <c r="S55" s="8" t="n"/>
+      <c r="S55" s="8" t="n">
+        <v>5280</v>
+      </c>
       <c r="T55" s="8" t="n"/>
       <c r="U55" s="8" t="n">
         <v>220</v>
@@ -6725,9 +6951,15 @@
         </is>
       </c>
       <c r="W55" s="8" t="n"/>
-      <c r="X55" s="8" t="n"/>
-      <c r="Y55" s="8" t="n"/>
-      <c r="Z55" s="8" t="n"/>
+      <c r="X55" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y55" s="8" t="n">
+        <v>792</v>
+      </c>
+      <c r="Z55" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA55" s="8" t="n"/>
       <c r="AB55" s="8" t="inlineStr">
         <is>
@@ -6761,7 +6993,7 @@
       <c r="AW55" s="8" t="n"/>
       <c r="AX55" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 792.0 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -6830,7 +7062,9 @@
       <c r="P56" s="8" t="n"/>
       <c r="Q56" s="8" t="n"/>
       <c r="R56" s="8" t="n"/>
-      <c r="S56" s="8" t="n"/>
+      <c r="S56" s="8" t="n">
+        <v>5280</v>
+      </c>
       <c r="T56" s="8" t="n"/>
       <c r="U56" s="8" t="n">
         <v>220</v>
@@ -6841,9 +7075,15 @@
         </is>
       </c>
       <c r="W56" s="8" t="n"/>
-      <c r="X56" s="8" t="n"/>
-      <c r="Y56" s="8" t="n"/>
-      <c r="Z56" s="8" t="n"/>
+      <c r="X56" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y56" s="8" t="n">
+        <v>792</v>
+      </c>
+      <c r="Z56" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA56" s="8" t="n"/>
       <c r="AB56" s="8" t="inlineStr">
         <is>
@@ -6877,7 +7117,7 @@
       <c r="AW56" s="8" t="n"/>
       <c r="AX56" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 792.0 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -6946,7 +7186,9 @@
       <c r="P57" s="8" t="n"/>
       <c r="Q57" s="8" t="n"/>
       <c r="R57" s="8" t="n"/>
-      <c r="S57" s="8" t="n"/>
+      <c r="S57" s="8" t="n">
+        <v>456</v>
+      </c>
       <c r="T57" s="8" t="n"/>
       <c r="U57" s="8" t="n">
         <v>19</v>
@@ -6957,9 +7199,15 @@
         </is>
       </c>
       <c r="W57" s="8" t="n"/>
-      <c r="X57" s="8" t="n"/>
-      <c r="Y57" s="8" t="n"/>
-      <c r="Z57" s="8" t="n"/>
+      <c r="X57" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y57" s="8" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="Z57" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA57" s="8" t="n"/>
       <c r="AB57" s="8" t="inlineStr">
         <is>
@@ -6993,7 +7241,7 @@
       <c r="AW57" s="8" t="n"/>
       <c r="AX57" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 68.4 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -7058,7 +7306,9 @@
       <c r="P58" s="8" t="n"/>
       <c r="Q58" s="8" t="n"/>
       <c r="R58" s="8" t="n"/>
-      <c r="S58" s="8" t="n"/>
+      <c r="S58" s="8" t="n">
+        <v>800</v>
+      </c>
       <c r="T58" s="8" t="n"/>
       <c r="U58" s="8" t="n">
         <v>20</v>
@@ -7069,9 +7319,15 @@
         </is>
       </c>
       <c r="W58" s="8" t="n"/>
-      <c r="X58" s="8" t="n"/>
-      <c r="Y58" s="8" t="n"/>
-      <c r="Z58" s="8" t="n"/>
+      <c r="X58" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y58" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="Z58" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA58" s="8" t="n"/>
       <c r="AB58" s="8" t="inlineStr">
         <is>
@@ -7105,7 +7361,7 @@
       <c r="AW58" s="8" t="n"/>
       <c r="AX58" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 120.0 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7430,9 @@
       <c r="P59" s="8" t="n"/>
       <c r="Q59" s="8" t="n"/>
       <c r="R59" s="8" t="n"/>
-      <c r="S59" s="8" t="n"/>
+      <c r="S59" s="8" t="n">
+        <v>3720</v>
+      </c>
       <c r="T59" s="8" t="n"/>
       <c r="U59" s="8" t="n">
         <v>155</v>
@@ -7185,9 +7443,15 @@
         </is>
       </c>
       <c r="W59" s="8" t="n"/>
-      <c r="X59" s="8" t="n"/>
-      <c r="Y59" s="8" t="n"/>
-      <c r="Z59" s="8" t="n"/>
+      <c r="X59" s="8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Y59" s="8" t="n">
+        <v>558</v>
+      </c>
+      <c r="Z59" s="8" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA59" s="8" t="n"/>
       <c r="AB59" s="8" t="inlineStr">
         <is>
@@ -7221,7 +7485,7 @@
       <c r="AW59" s="8" t="n"/>
       <c r="AX59" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 558.0 kg CO₂e (UltraTech Cement plaster EPD; density from IS 2250).</t>
         </is>
       </c>
     </row>
@@ -8076,7 +8340,9 @@
       <c r="P67" s="8" t="n"/>
       <c r="Q67" s="8" t="n"/>
       <c r="R67" s="8" t="n"/>
-      <c r="S67" s="8" t="n"/>
+      <c r="S67" s="8" t="n">
+        <v>5951.25</v>
+      </c>
       <c r="T67" s="8" t="n"/>
       <c r="U67" s="8" t="n">
         <v>34.5</v>
@@ -8087,9 +8353,15 @@
         </is>
       </c>
       <c r="W67" s="8" t="n"/>
-      <c r="X67" s="8" t="n"/>
-      <c r="Y67" s="8" t="n"/>
-      <c r="Z67" s="8" t="n"/>
+      <c r="X67" s="8" t="n">
+        <v>2300</v>
+      </c>
+      <c r="Y67" s="8" t="n">
+        <v>595.12</v>
+      </c>
+      <c r="Z67" s="8" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AA67" s="8" t="n"/>
       <c r="AB67" s="8" t="inlineStr">
         <is>
@@ -8123,7 +8395,7 @@
       <c r="AW67" s="8" t="n"/>
       <c r="AX67" s="8" t="inlineStr">
         <is>
-          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields.</t>
+          <t>[OCR] Extracted from scanned BoQ; manual review applied to low-legibility fields. | [Carbon] EPD-backed estimate: 595.12 kg CO₂e (ACC Cement concrete EPD; density from IS 456).</t>
         </is>
       </c>
     </row>

</xml_diff>